<commit_message>
modif societe sans actions
</commit_message>
<xml_diff>
--- a/public/docs/exemplaires-import-biens/exemplaire_immeubles.xlsx
+++ b/public/docs/exemplaires-import-biens/exemplaire_immeubles.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D9EDA3D-82AA-4D82-B335-4C9C78D497CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5196"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -19,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="38">
-  <si>
-    <t>RDC</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Immeuble</t>
   </si>
@@ -112,34 +110,13 @@
   </si>
   <si>
     <t>Nombre facade</t>
-  </si>
-  <si>
-    <t>imm09</t>
-  </si>
-  <si>
-    <t>imm10</t>
-  </si>
-  <si>
-    <t>B33_9</t>
-  </si>
-  <si>
-    <t>B34_10</t>
-  </si>
-  <si>
-    <t>B35_10</t>
-  </si>
-  <si>
-    <t>1er etage</t>
-  </si>
-  <si>
-    <t>15</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,15 +132,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -176,70 +146,11 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="4">
+  <borders count="1">
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="hair">
-        <color auto="1"/>
-      </right>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="hair">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="hair">
-        <color auto="1"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -248,32 +159,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,267 +441,126 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AD1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="8.88671875" customWidth="1"/>
+    <col min="2" max="2" width="8.90625" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="22.88671875" customWidth="1"/>
-    <col min="7" max="7" width="21.77734375" customWidth="1"/>
-    <col min="8" max="8" width="23.33203125" customWidth="1"/>
+    <col min="6" max="6" width="22.90625" customWidth="1"/>
+    <col min="7" max="7" width="21.81640625" customWidth="1"/>
+    <col min="8" max="8" width="23.36328125" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="12.77734375" customWidth="1"/>
+    <col min="11" max="11" width="12.81640625" customWidth="1"/>
     <col min="12" max="12" width="19" customWidth="1"/>
-    <col min="13" max="13" width="19.21875" customWidth="1"/>
-    <col min="14" max="14" width="17.5546875" customWidth="1"/>
-    <col min="15" max="15" width="16.21875" customWidth="1"/>
-    <col min="16" max="16" width="14.21875" customWidth="1"/>
-    <col min="17" max="17" width="12.109375" customWidth="1"/>
-    <col min="18" max="18" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.1796875" customWidth="1"/>
+    <col min="14" max="14" width="17.54296875" customWidth="1"/>
+    <col min="15" max="15" width="16.1796875" customWidth="1"/>
+    <col min="16" max="16" width="14.1796875" customWidth="1"/>
+    <col min="17" max="17" width="12.08984375" customWidth="1"/>
+    <col min="18" max="18" width="15.08984375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="18" customWidth="1"/>
-    <col min="20" max="20" width="18.5546875" customWidth="1"/>
+    <col min="20" max="20" width="18.54296875" customWidth="1"/>
     <col min="21" max="21" width="19" customWidth="1"/>
-    <col min="22" max="23" width="17.88671875" customWidth="1"/>
+    <col min="22" max="23" width="17.90625" customWidth="1"/>
     <col min="24" max="25" width="19" customWidth="1"/>
-    <col min="26" max="28" width="17.88671875" customWidth="1"/>
+    <col min="26" max="28" width="17.90625" customWidth="1"/>
     <col min="29" max="29" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="X1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:30" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" s="2">
-        <v>0</v>
-      </c>
-      <c r="F2" s="2">
-        <v>60</v>
-      </c>
-      <c r="G2" s="4">
-        <v>4</v>
-      </c>
-      <c r="H2" s="4"/>
-      <c r="J2" s="9">
-        <v>88888</v>
-      </c>
-      <c r="K2" s="9">
-        <v>45000</v>
-      </c>
-      <c r="M2" s="10">
-        <v>2</v>
-      </c>
-      <c r="N2" s="10">
-        <v>1</v>
-      </c>
-      <c r="O2" s="10">
-        <v>1</v>
-      </c>
-      <c r="P2" s="10">
-        <v>2</v>
-      </c>
-      <c r="T2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:30" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E3" s="12">
-        <v>30</v>
-      </c>
-      <c r="F3" s="12">
-        <v>0</v>
-      </c>
-      <c r="G3" s="7">
-        <v>4</v>
-      </c>
-      <c r="H3" s="7"/>
-      <c r="J3" s="11">
-        <v>11800</v>
-      </c>
-      <c r="K3" s="11">
-        <v>45000</v>
-      </c>
-      <c r="M3" s="10">
-        <v>2</v>
-      </c>
-      <c r="N3" s="10">
-        <v>1</v>
-      </c>
-      <c r="O3" s="10">
-        <v>1</v>
-      </c>
-      <c r="P3" s="10">
-        <v>2</v>
-      </c>
-      <c r="T3">
-        <v>1</v>
-      </c>
-      <c r="U3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" s="12">
-        <v>820</v>
-      </c>
-      <c r="F4" s="12">
-        <v>0</v>
-      </c>
-      <c r="G4" s="7">
-        <v>4</v>
-      </c>
-      <c r="H4" s="7"/>
-      <c r="J4" s="11">
-        <v>11800</v>
-      </c>
-      <c r="K4" s="11">
-        <v>45000</v>
-      </c>
-      <c r="M4" s="10">
-        <v>2</v>
-      </c>
-      <c r="N4" s="10">
-        <v>1</v>
-      </c>
-      <c r="O4" s="10">
-        <v>1</v>
-      </c>
-      <c r="P4" s="10">
-        <v>2</v>
-      </c>
-      <c r="T4">
-        <v>1</v>
-      </c>
-      <c r="U4">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>